<commit_message>
Run full flow from: Login Admin Page > Add Brand > Add Category > Add Product && Check detail của 1 product vừa add trong Admin Page với thông tin bên ngoài trang User Page (View Product)
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/logindata.xlsx
+++ b/src/test/resources/testdata/logindata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tester\Automation\Hoa_Baitapcuoikhoa_AT04\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E47E8B-119B-4A8B-8AB5-0CA4C8A952FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B111EE-B97F-436F-9F2E-E28F8FCED427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2385" yWindow="4095" windowWidth="14595" windowHeight="11385" activeTab="2" xr2:uid="{6A5B7545-1E47-48FC-9C01-3B596E42F566}"/>
+    <workbookView xWindow="1080" yWindow="4215" windowWidth="14595" windowHeight="11385" activeTab="2" xr2:uid="{6A5B7545-1E47-48FC-9C01-3B596E42F566}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -130,9 +130,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>My Pham</t>
-  </si>
-  <si>
     <t>Chanel</t>
   </si>
   <si>
@@ -142,12 +139,6 @@
     <t>Dior</t>
   </si>
   <si>
-    <t>Phu Kien</t>
-  </si>
-  <si>
-    <t>Trang suc</t>
-  </si>
-  <si>
     <t>PNJ</t>
   </si>
   <si>
@@ -191,6 +182,15 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>Category 1</t>
+  </si>
+  <si>
+    <t>Mỹ Phẩm</t>
+  </si>
+  <si>
+    <t>Cake</t>
   </si>
 </sst>
 </file>
@@ -686,16 +686,16 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="C2">
         <v>1000</v>
       </c>
       <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
         <v>30</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -703,16 +703,16 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>1011</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -720,16 +720,16 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C4">
         <v>1021</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -753,28 +753,28 @@
         <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
-        <v>42</v>
-      </c>
       <c r="F1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
-        <v>47</v>
-      </c>
       <c r="I1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="J1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -782,13 +782,13 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E2">
         <v>0.8</v>
@@ -797,7 +797,7 @@
         <v>200</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H2">
         <v>4000</v>
@@ -814,13 +814,13 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E3">
         <v>3.2</v>
@@ -829,7 +829,7 @@
         <v>500</v>
       </c>
       <c r="G3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H3">
         <v>5000</v>

</xml_diff>